<commit_message>
Atualização automática de dados local - 23/06/2026 13:50
</commit_message>
<xml_diff>
--- a/planilhas_para_atualizar/f_rodadas_ampere.xlsx
+++ b/planilhas_para_atualizar/f_rodadas_ampere.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1661"/>
+  <dimension ref="A1:M1729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85147,6 +85147,3474 @@
         <v>46189</v>
       </c>
     </row>
+    <row r="1662">
+      <c r="A1662" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1662" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1662" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1662" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1662" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1662" t="n">
+        <v>29794</v>
+      </c>
+      <c r="G1662" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1662" t="inlineStr"/>
+      <c r="I1662" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1662" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1662" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1662" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1662" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1663" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1663" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1663" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1663" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1663" t="n">
+        <v>92</v>
+      </c>
+      <c r="G1663" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1663" t="inlineStr"/>
+      <c r="I1663" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1663" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1663" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1663" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1663" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1664" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1664" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1664" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1664" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1664" t="n">
+        <v>23110</v>
+      </c>
+      <c r="G1664" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1664" t="inlineStr"/>
+      <c r="I1664" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1664" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1664" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1664" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1664" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1665" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1665" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1665" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1665" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1665" t="n">
+        <v>91</v>
+      </c>
+      <c r="G1665" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1665" t="inlineStr"/>
+      <c r="I1665" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1665" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1665" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1665" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1665" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1666" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1666" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1666" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1666" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1666" t="n">
+        <v>18779</v>
+      </c>
+      <c r="G1666" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1666" t="inlineStr"/>
+      <c r="I1666" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1666" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1666" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1666" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1666" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1667" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1667" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1667" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1667" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1667" t="n">
+        <v>92</v>
+      </c>
+      <c r="G1667" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1667" t="inlineStr"/>
+      <c r="I1667" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1667" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1667" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1667" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1667" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1668" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1668" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1668" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1668" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1668" t="n">
+        <v>16987</v>
+      </c>
+      <c r="G1668" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1668" t="inlineStr"/>
+      <c r="I1668" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1668" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1668" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1668" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1668" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1669" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1669" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1669" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1669" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1669" t="n">
+        <v>87</v>
+      </c>
+      <c r="G1669" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1669" t="inlineStr"/>
+      <c r="I1669" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1669" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1669" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1669" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1669" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1670" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1670" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1670" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1670" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1670" t="n">
+        <v>6859</v>
+      </c>
+      <c r="G1670" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1670" t="inlineStr"/>
+      <c r="I1670" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1670" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1670" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1670" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1670" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1671" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1671" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1671" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1671" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1671" t="n">
+        <v>64</v>
+      </c>
+      <c r="G1671" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1671" t="inlineStr"/>
+      <c r="I1671" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1671" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1671" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1671" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1671" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1672" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1672" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1672" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1672" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1672" t="n">
+        <v>10437</v>
+      </c>
+      <c r="G1672" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1672" t="inlineStr"/>
+      <c r="I1672" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1672" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1672" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1672" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1672" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1673" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1673" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1673" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1673" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1673" t="n">
+        <v>94</v>
+      </c>
+      <c r="G1673" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1673" t="inlineStr"/>
+      <c r="I1673" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1673" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1673" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1673" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1673" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1674" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1674" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1674" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1674" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1674" t="n">
+        <v>10718</v>
+      </c>
+      <c r="G1674" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1674" t="inlineStr"/>
+      <c r="I1674" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1674" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1674" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1674" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1674" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1675" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1675" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1675" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1675" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1675" t="n">
+        <v>108</v>
+      </c>
+      <c r="G1675" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1675" t="inlineStr"/>
+      <c r="I1675" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1675" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1675" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1675" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1675" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1676" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1676" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1676" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1676" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1676" t="n">
+        <v>16440</v>
+      </c>
+      <c r="G1676" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1676" t="inlineStr"/>
+      <c r="I1676" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1676" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1676" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1676" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1676" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1677" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1677" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1677" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1677" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1677" t="n">
+        <v>141</v>
+      </c>
+      <c r="G1677" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1677" t="inlineStr"/>
+      <c r="I1677" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1677" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1677" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1677" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1677" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1678" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1678" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1678" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1678" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1678" t="n">
+        <v>2587</v>
+      </c>
+      <c r="G1678" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1678" t="inlineStr"/>
+      <c r="I1678" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1678" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1678" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1678" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1678" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1679" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1679" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1679" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1679" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1679" t="n">
+        <v>57</v>
+      </c>
+      <c r="G1679" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1679" t="inlineStr"/>
+      <c r="I1679" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1679" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1679" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1679" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1679" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1680" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1680" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1680" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1680" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1680" t="n">
+        <v>2334</v>
+      </c>
+      <c r="G1680" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1680" t="inlineStr"/>
+      <c r="I1680" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1680" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1680" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1680" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1680" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1681" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1681" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1681" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1681" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1681" t="n">
+        <v>63</v>
+      </c>
+      <c r="G1681" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1681" t="inlineStr"/>
+      <c r="I1681" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1681" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1681" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1681" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1681" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1682" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1682" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1682" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1682" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1682" t="n">
+        <v>2096</v>
+      </c>
+      <c r="G1682" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1682" t="inlineStr"/>
+      <c r="I1682" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1682" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1682" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1682" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1682" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1683" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1683" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1683" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1683" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1683" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1683" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1683" t="inlineStr"/>
+      <c r="I1683" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1683" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1683" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1683" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1683" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1684" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1684" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1684" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1684" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1684" t="n">
+        <v>1935</v>
+      </c>
+      <c r="G1684" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1684" t="inlineStr"/>
+      <c r="I1684" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1684" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1684" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1684" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1684" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1685" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1685" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1685" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1685" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1685" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1685" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1685" t="inlineStr"/>
+      <c r="I1685" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1685" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1685" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1685" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1685" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1686" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1686" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1686" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1686" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1686" t="n">
+        <v>6498</v>
+      </c>
+      <c r="G1686" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1686" t="inlineStr"/>
+      <c r="I1686" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1686" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1686" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1686" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1686" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1687" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1687" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1687" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1687" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1687" t="n">
+        <v>61</v>
+      </c>
+      <c r="G1687" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1687" t="inlineStr"/>
+      <c r="I1687" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1687" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1687" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1687" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1687" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1688" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1688" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1688" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1688" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1688" t="n">
+        <v>3616</v>
+      </c>
+      <c r="G1688" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1688" t="inlineStr"/>
+      <c r="I1688" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1688" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1688" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1688" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1688" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1689" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1689" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1689" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1689" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1689" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1689" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1689" t="inlineStr"/>
+      <c r="I1689" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1689" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1689" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1689" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1689" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1690" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1690" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1690" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1690" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1690" t="n">
+        <v>2176</v>
+      </c>
+      <c r="G1690" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1690" t="inlineStr"/>
+      <c r="I1690" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1690" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1690" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1690" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1690" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1691" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1691" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1691" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1691" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1691" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1691" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1691" t="inlineStr"/>
+      <c r="I1691" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1691" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1691" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1691" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1691" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1692" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1692" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1692" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1692" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1692" t="n">
+        <v>1396</v>
+      </c>
+      <c r="G1692" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1692" t="inlineStr"/>
+      <c r="I1692" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1692" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1692" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1692" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1692" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1693" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1693" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1693" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1693" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1693" t="n">
+        <v>62</v>
+      </c>
+      <c r="G1693" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1693" t="inlineStr"/>
+      <c r="I1693" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1693" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1693" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1693" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1693" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1694" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1694" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1694" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1694" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1694" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="G1694" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1694" t="inlineStr"/>
+      <c r="I1694" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1694" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1694" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1694" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1694" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1695" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1695" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1695" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1695" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1695" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="G1695" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1695" t="inlineStr"/>
+      <c r="I1695" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1695" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1695" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1695" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1695" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1696" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1696" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1696" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1696" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1696" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="G1696" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1696" t="inlineStr"/>
+      <c r="I1696" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1696" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1696" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1696" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1696" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1697" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1697" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1697" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1697" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1697" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="G1697" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1697" t="inlineStr"/>
+      <c r="I1697" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1697" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1697" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1697" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1697" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1698" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1698" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1698" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1698" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1698" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="G1698" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1698" t="inlineStr"/>
+      <c r="I1698" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1698" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1698" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1698" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1698" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1699" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1699" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1699" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1699" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1699" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="G1699" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1699" t="inlineStr"/>
+      <c r="I1699" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1699" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1699" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1699" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1699" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1700" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1700" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1700" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1700" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1700" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="G1700" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1700" t="inlineStr"/>
+      <c r="I1700" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1700" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1700" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1700" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1700" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1701" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1701" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1701" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1701" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1701" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="G1701" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1701" t="inlineStr"/>
+      <c r="I1701" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1701" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1701" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1701" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1701" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1702" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1702" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1702" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1702" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1702" t="n">
+        <v>89</v>
+      </c>
+      <c r="G1702" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1702" t="inlineStr"/>
+      <c r="I1702" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1702" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1702" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1702" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1702" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1703" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1703" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1703" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1703" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1703" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="G1703" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1703" t="inlineStr"/>
+      <c r="I1703" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1703" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1703" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1703" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1703" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1704" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1704" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1704" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1704" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1704" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="G1704" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1704" t="inlineStr"/>
+      <c r="I1704" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1704" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1704" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1704" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1704" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1705" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1705" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1705" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1705" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1705" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="G1705" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1705" t="inlineStr"/>
+      <c r="I1705" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1705" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1705" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1705" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1705" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1706" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1706" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1706" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1706" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1706" t="n">
+        <v>93.8</v>
+      </c>
+      <c r="G1706" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1706" t="inlineStr"/>
+      <c r="I1706" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1706" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1706" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1706" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1706" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1707" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1707" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1707" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1707" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1707" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="G1707" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1707" t="inlineStr"/>
+      <c r="I1707" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1707" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1707" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1707" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1707" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1708" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1708" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1708" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1708" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1708" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="G1708" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1708" t="inlineStr"/>
+      <c r="I1708" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1708" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1708" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1708" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1708" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1709" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1709" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1709" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1709" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1709" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="G1709" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1709" t="inlineStr"/>
+      <c r="I1709" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1709" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1709" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1709" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1709" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1710" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1710" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1710" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1710" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1710" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="G1710" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1710" t="inlineStr"/>
+      <c r="I1710" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1710" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1710" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1710" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1710" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1711" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1711" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1711" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1711" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1711" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="G1711" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1711" t="inlineStr"/>
+      <c r="I1711" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1711" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1711" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1711" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1711" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1712" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1712" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1712" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1712" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1712" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="G1712" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1712" t="inlineStr"/>
+      <c r="I1712" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1712" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1712" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1712" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1712" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1713" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1713" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1713" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1713" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1713" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="G1713" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1713" t="inlineStr"/>
+      <c r="I1713" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1713" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1713" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1713" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1713" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1714" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1714" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1714" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1714" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1714" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="G1714" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1714" t="inlineStr"/>
+      <c r="I1714" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1714" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1714" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1714" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1714" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1715" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1715" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1715" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1715" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1715" t="n">
+        <v>179.97</v>
+      </c>
+      <c r="G1715" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1715" t="inlineStr"/>
+      <c r="I1715" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1715" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1715" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1715" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1715" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1716" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1716" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1716" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1716" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1716" t="n">
+        <v>161.46</v>
+      </c>
+      <c r="G1716" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1716" t="inlineStr"/>
+      <c r="I1716" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1716" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1716" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1716" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1716" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1717" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1717" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1717" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1717" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1717" t="n">
+        <v>169.86</v>
+      </c>
+      <c r="G1717" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1717" t="inlineStr"/>
+      <c r="I1717" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1717" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1717" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1717" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1717" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1718" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1718" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1718" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1718" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1718" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="G1718" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1718" t="inlineStr"/>
+      <c r="I1718" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1718" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1718" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1718" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1718" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1719" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1719" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1719" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1719" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1719" t="n">
+        <v>179.97</v>
+      </c>
+      <c r="G1719" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1719" t="inlineStr"/>
+      <c r="I1719" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1719" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1719" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1719" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1719" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1720" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1720" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1720" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1720" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1720" t="n">
+        <v>161.46</v>
+      </c>
+      <c r="G1720" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1720" t="inlineStr"/>
+      <c r="I1720" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1720" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1720" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1720" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1720" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1721" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1721" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1721" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1721" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1721" t="n">
+        <v>169.86</v>
+      </c>
+      <c r="G1721" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1721" t="inlineStr"/>
+      <c r="I1721" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1721" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1721" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1721" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1721" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1722" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1722" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1722" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1722" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1722" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="G1722" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1722" t="inlineStr"/>
+      <c r="I1722" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1722" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1722" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1722" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1722" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1723" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1723" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1723" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1723" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1723" t="n">
+        <v>179.97</v>
+      </c>
+      <c r="G1723" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1723" t="inlineStr"/>
+      <c r="I1723" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1723" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1723" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1723" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1723" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1724" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1724" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1724" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1724" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1724" t="n">
+        <v>161.46</v>
+      </c>
+      <c r="G1724" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1724" t="inlineStr"/>
+      <c r="I1724" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1724" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1724" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1724" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1724" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1725" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1725" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1725" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1725" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1725" t="n">
+        <v>169.8</v>
+      </c>
+      <c r="G1725" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1725" t="inlineStr"/>
+      <c r="I1725" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1725" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1725" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1725" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1725" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1726" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1726" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1726" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1726" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1726" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="G1726" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1726" t="inlineStr"/>
+      <c r="I1726" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1726" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1726" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1726" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1726" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1727" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1727" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1727" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1727" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1727" t="n">
+        <v>179.97</v>
+      </c>
+      <c r="G1727" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1727" t="inlineStr"/>
+      <c r="I1727" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1727" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1727" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1727" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1727" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1728" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1728" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1728" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1728" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1728" t="n">
+        <v>161.46</v>
+      </c>
+      <c r="G1728" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1728" t="inlineStr"/>
+      <c r="I1728" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1728" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1728" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1728" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1728" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1729" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1729" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1729" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1729" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1729" t="n">
+        <v>169.86</v>
+      </c>
+      <c r="G1729" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1729" t="inlineStr"/>
+      <c r="I1729" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1729" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1729" t="n">
+        <v>20260623</v>
+      </c>
+      <c r="L1729" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1729" s="1" t="n">
+        <v>46196</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização do relatório Ampere - Rodada 30/06/2026
</commit_message>
<xml_diff>
--- a/planilhas_para_atualizar/f_rodadas_ampere.xlsx
+++ b/planilhas_para_atualizar/f_rodadas_ampere.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1729"/>
+  <dimension ref="A1:M1797"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -88615,6 +88615,3474 @@
         <v>46196</v>
       </c>
     </row>
+    <row r="1730">
+      <c r="A1730" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1730" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1730" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1730" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1730" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1730" t="n">
+        <v>25564</v>
+      </c>
+      <c r="G1730" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1730" t="inlineStr"/>
+      <c r="I1730" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1730" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1730" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1730" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1730" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1731" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1731" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1731" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1731" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1731" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1731" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1731" t="inlineStr"/>
+      <c r="I1731" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1731" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1731" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1731" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1731" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1732" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1732" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1732" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1732" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1732" t="n">
+        <v>20775</v>
+      </c>
+      <c r="G1732" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1732" t="inlineStr"/>
+      <c r="I1732" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1732" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1732" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1732" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1732" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1733" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1733" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1733" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1733" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1733" t="n">
+        <v>101</v>
+      </c>
+      <c r="G1733" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1733" t="inlineStr"/>
+      <c r="I1733" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1733" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1733" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1733" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1733" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1734" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1734" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1734" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1734" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1734" t="n">
+        <v>18383</v>
+      </c>
+      <c r="G1734" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1734" t="inlineStr"/>
+      <c r="I1734" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1734" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1734" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1734" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1734" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1735" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1735" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1735" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1735" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1735" t="n">
+        <v>94</v>
+      </c>
+      <c r="G1735" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1735" t="inlineStr"/>
+      <c r="I1735" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1735" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1735" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1735" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1735" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1736" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1736" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1736" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1736" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1736" t="n">
+        <v>19884</v>
+      </c>
+      <c r="G1736" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1736" t="inlineStr"/>
+      <c r="I1736" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1736" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1736" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1736" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1736" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1737" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1737" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1737" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1737" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1737" t="n">
+        <v>84</v>
+      </c>
+      <c r="G1737" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1737" t="inlineStr"/>
+      <c r="I1737" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1737" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1737" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1737" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1737" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1738" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1738" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1738" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1738" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1738" t="n">
+        <v>19265</v>
+      </c>
+      <c r="G1738" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1738" t="inlineStr"/>
+      <c r="I1738" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1738" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1738" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1738" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1738" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1739" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1739" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1739" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1739" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1739" t="n">
+        <v>174</v>
+      </c>
+      <c r="G1739" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1739" t="inlineStr"/>
+      <c r="I1739" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1739" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1739" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1739" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1739" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1740" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1740" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1740" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1740" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1740" t="n">
+        <v>14970</v>
+      </c>
+      <c r="G1740" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1740" t="inlineStr"/>
+      <c r="I1740" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1740" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1740" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1740" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1740" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1741" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1741" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1741" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1741" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1741" t="n">
+        <v>151</v>
+      </c>
+      <c r="G1741" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1741" t="inlineStr"/>
+      <c r="I1741" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1741" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1741" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1741" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1741" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1742" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1742" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1742" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1742" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1742" t="n">
+        <v>17244</v>
+      </c>
+      <c r="G1742" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1742" t="inlineStr"/>
+      <c r="I1742" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1742" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1742" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1742" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1742" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1743" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1743" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1743" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1743" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1743" t="n">
+        <v>148</v>
+      </c>
+      <c r="G1743" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1743" t="inlineStr"/>
+      <c r="I1743" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1743" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1743" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1743" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1743" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1744" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1744" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1744" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1744" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1744" t="n">
+        <v>33844</v>
+      </c>
+      <c r="G1744" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1744" t="inlineStr"/>
+      <c r="I1744" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1744" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1744" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1744" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1744" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1745" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1745" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1745" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1745" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1745" t="n">
+        <v>247</v>
+      </c>
+      <c r="G1745" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1745" t="inlineStr"/>
+      <c r="I1745" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1745" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1745" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1745" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1745" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1746" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1746" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1746" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1746" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1746" t="n">
+        <v>2311</v>
+      </c>
+      <c r="G1746" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1746" t="inlineStr"/>
+      <c r="I1746" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1746" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1746" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1746" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1746" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1747" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1747" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1747" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1747" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1747" t="n">
+        <v>62</v>
+      </c>
+      <c r="G1747" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1747" t="inlineStr"/>
+      <c r="I1747" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1747" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1747" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1747" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1747" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1748" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1748" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1748" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1748" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1748" t="n">
+        <v>2086</v>
+      </c>
+      <c r="G1748" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1748" t="inlineStr"/>
+      <c r="I1748" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1748" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1748" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1748" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1748" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1749" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1749" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1749" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1749" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1749" t="n">
+        <v>64</v>
+      </c>
+      <c r="G1749" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1749" t="inlineStr"/>
+      <c r="I1749" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1749" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1749" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1749" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1749" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1750" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1750" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1750" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1750" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1750" t="n">
+        <v>1916</v>
+      </c>
+      <c r="G1750" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1750" t="inlineStr"/>
+      <c r="I1750" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1750" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1750" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1750" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1750" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1751" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1751" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1751" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1751" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1751" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1751" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1751" t="inlineStr"/>
+      <c r="I1751" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1751" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1751" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1751" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1751" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1752" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1752" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1752" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1752" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1752" t="n">
+        <v>1601</v>
+      </c>
+      <c r="G1752" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1752" t="inlineStr"/>
+      <c r="I1752" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1752" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1752" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1752" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1752" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1753" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1753" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1753" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1753" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1753" t="n">
+        <v>51</v>
+      </c>
+      <c r="G1753" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1753" t="inlineStr"/>
+      <c r="I1753" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1753" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1753" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1753" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1753" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1754" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1754" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1754" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1754" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1754" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G1754" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1754" t="inlineStr"/>
+      <c r="I1754" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1754" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1754" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1754" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1754" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1755" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1755" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1755" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1755" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1755" t="n">
+        <v>65</v>
+      </c>
+      <c r="G1755" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1755" t="inlineStr"/>
+      <c r="I1755" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1755" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1755" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1755" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1755" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1756" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1756" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1756" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1756" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1756" t="n">
+        <v>2004</v>
+      </c>
+      <c r="G1756" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1756" t="inlineStr"/>
+      <c r="I1756" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1756" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1756" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1756" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1756" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1757" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1757" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1757" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1757" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1757" t="n">
+        <v>63</v>
+      </c>
+      <c r="G1757" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1757" t="inlineStr"/>
+      <c r="I1757" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1757" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1757" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1757" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1757" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1758" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1758" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1758" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1758" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1758" t="n">
+        <v>1291</v>
+      </c>
+      <c r="G1758" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1758" t="inlineStr"/>
+      <c r="I1758" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1758" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1758" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1758" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1758" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1759" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1759" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1759" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1759" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1759" t="n">
+        <v>57</v>
+      </c>
+      <c r="G1759" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1759" t="inlineStr"/>
+      <c r="I1759" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1759" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1759" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1759" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1759" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1760" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1760" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1760" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1760" t="inlineStr">
+        <is>
+          <t>MWmed</t>
+        </is>
+      </c>
+      <c r="F1760" t="n">
+        <v>909</v>
+      </c>
+      <c r="G1760" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1760" t="inlineStr"/>
+      <c r="I1760" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1760" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1760" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1760" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1760" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1761" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1761" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1761" t="inlineStr">
+        <is>
+          <t>ENA</t>
+        </is>
+      </c>
+      <c r="E1761" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1761" t="n">
+        <v>39</v>
+      </c>
+      <c r="G1761" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1761" t="inlineStr"/>
+      <c r="I1761" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1761" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1761" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1761" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1761" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1762" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1762" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1762" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1762" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1762" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1762" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1762" t="inlineStr"/>
+      <c r="I1762" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1762" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1762" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1762" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1762" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1763" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1763" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1763" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1763" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1763" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="G1763" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1763" t="inlineStr"/>
+      <c r="I1763" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1763" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1763" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1763" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1763" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1764" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1764" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1764" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1764" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1764" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="G1764" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1764" t="inlineStr"/>
+      <c r="I1764" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1764" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1764" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1764" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1764" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1765" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1765" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1765" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1765" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1765" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="G1765" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1765" t="inlineStr"/>
+      <c r="I1765" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1765" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1765" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1765" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1765" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1766" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1766" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1766" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1766" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1766" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="G1766" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1766" t="inlineStr"/>
+      <c r="I1766" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1766" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1766" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1766" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1766" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1767" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1767" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1767" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1767" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1767" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="G1767" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1767" t="inlineStr"/>
+      <c r="I1767" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1767" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1767" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1767" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1767" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1768" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1768" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1768" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1768" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1768" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="G1768" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1768" t="inlineStr"/>
+      <c r="I1768" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1768" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1768" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1768" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1768" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1769" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1769" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1769" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1769" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1769" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="G1769" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1769" t="inlineStr"/>
+      <c r="I1769" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1769" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1769" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1769" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1769" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1770" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1770" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1770" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1770" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1770" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="G1770" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1770" t="inlineStr"/>
+      <c r="I1770" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1770" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1770" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1770" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1770" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1771" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1771" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1771" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1771" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1771" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="G1771" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1771" t="inlineStr"/>
+      <c r="I1771" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1771" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1771" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1771" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1771" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1772" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1772" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1772" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1772" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1772" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="G1772" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1772" t="inlineStr"/>
+      <c r="I1772" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1772" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1772" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1772" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1772" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1773" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1773" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1773" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1773" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1773" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="G1773" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1773" t="inlineStr"/>
+      <c r="I1773" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1773" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1773" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1773" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1773" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1774" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1774" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1774" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1774" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1774" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="G1774" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1774" t="inlineStr"/>
+      <c r="I1774" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1774" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1774" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1774" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1774" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1775" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1775" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1775" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1775" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1775" t="n">
+        <v>92.2</v>
+      </c>
+      <c r="G1775" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1775" t="inlineStr"/>
+      <c r="I1775" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1775" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1775" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1775" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1775" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1776" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1776" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1776" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1776" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1776" t="n">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="G1776" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1776" t="inlineStr"/>
+      <c r="I1776" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1776" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1776" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1776" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1776" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1777" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1777" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1777" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1777" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1777" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="G1777" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1777" t="inlineStr"/>
+      <c r="I1777" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1777" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1777" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1777" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1777" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1778" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1778" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1778" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1778" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1778" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="G1778" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1778" t="inlineStr"/>
+      <c r="I1778" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1778" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1778" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1778" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1778" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1779" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1779" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1779" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1779" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1779" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="G1779" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1779" t="inlineStr"/>
+      <c r="I1779" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1779" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1779" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1779" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1779" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1780" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1780" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1780" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1780" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1780" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1780" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1780" t="inlineStr"/>
+      <c r="I1780" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1780" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1780" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1780" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1780" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1781" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1781" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1781" t="inlineStr">
+        <is>
+          <t>Armazenamento</t>
+        </is>
+      </c>
+      <c r="E1781" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F1781" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="G1781" t="inlineStr">
+        <is>
+          <t>SIN</t>
+        </is>
+      </c>
+      <c r="H1781" t="inlineStr"/>
+      <c r="I1781" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1781" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1781" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1781" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1781" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1782" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1782" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1782" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1782" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1782" t="n">
+        <v>148.55</v>
+      </c>
+      <c r="G1782" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1782" t="inlineStr"/>
+      <c r="I1782" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1782" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1782" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1782" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1782" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1783" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1783" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1783" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1783" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1783" t="n">
+        <v>79.22</v>
+      </c>
+      <c r="G1783" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1783" t="inlineStr"/>
+      <c r="I1783" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1783" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1783" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1783" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1783" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1784" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1784" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1784" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1784" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1784" t="n">
+        <v>95.01000000000001</v>
+      </c>
+      <c r="G1784" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1784" t="inlineStr"/>
+      <c r="I1784" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1784" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1784" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1784" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1784" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1785" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1785" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1785" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1785" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1785" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1785" t="inlineStr">
+        <is>
+          <t>Sudeste/Centro-Oeste</t>
+        </is>
+      </c>
+      <c r="H1785" t="inlineStr"/>
+      <c r="I1785" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1785" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1785" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1785" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1785" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1786" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1786" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1786" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1786" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1786" t="n">
+        <v>148.55</v>
+      </c>
+      <c r="G1786" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1786" t="inlineStr"/>
+      <c r="I1786" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1786" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1786" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1786" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1786" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1787" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1787" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1787" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1787" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1787" t="n">
+        <v>79.22</v>
+      </c>
+      <c r="G1787" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1787" t="inlineStr"/>
+      <c r="I1787" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1787" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1787" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1787" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1787" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1788" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1788" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1788" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1788" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1788" t="n">
+        <v>95.01000000000001</v>
+      </c>
+      <c r="G1788" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1788" t="inlineStr"/>
+      <c r="I1788" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1788" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1788" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1788" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1788" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1789" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1789" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1789" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1789" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1789" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1789" t="inlineStr">
+        <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="H1789" t="inlineStr"/>
+      <c r="I1789" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1789" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1789" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1789" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1789" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1790" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1790" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1790" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1790" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1790" t="n">
+        <v>148.55</v>
+      </c>
+      <c r="G1790" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1790" t="inlineStr"/>
+      <c r="I1790" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1790" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1790" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1790" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1790" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1791" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1791" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1791" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1791" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1791" t="n">
+        <v>79.22</v>
+      </c>
+      <c r="G1791" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1791" t="inlineStr"/>
+      <c r="I1791" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1791" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1791" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1791" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1791" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1792" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1792" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1792" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1792" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1792" t="n">
+        <v>95.01000000000001</v>
+      </c>
+      <c r="G1792" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1792" t="inlineStr"/>
+      <c r="I1792" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1792" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1792" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1792" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1792" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1793" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1793" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1793" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1793" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1793" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1793" t="inlineStr">
+        <is>
+          <t>Nordeste</t>
+        </is>
+      </c>
+      <c r="H1793" t="inlineStr"/>
+      <c r="I1793" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1793" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1793" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1793" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1793" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1794" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1794" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1794" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1794" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1794" t="n">
+        <v>148.55</v>
+      </c>
+      <c r="G1794" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1794" t="inlineStr"/>
+      <c r="I1794" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1794" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1794" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1794" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1794" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B1795" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1795" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1795" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1795" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1795" t="n">
+        <v>79.22</v>
+      </c>
+      <c r="G1795" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1795" t="inlineStr"/>
+      <c r="I1795" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1795" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1795" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1795" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1795" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1796" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1796" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1796" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1796" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1796" t="n">
+        <v>95.01000000000001</v>
+      </c>
+      <c r="G1796" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1796" t="inlineStr"/>
+      <c r="I1796" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1796" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1796" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1796" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1796" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1797" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C1797" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1797" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="E1797" t="inlineStr">
+        <is>
+          <t>R$/MWh</t>
+        </is>
+      </c>
+      <c r="F1797" t="n">
+        <v>69</v>
+      </c>
+      <c r="G1797" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+      <c r="H1797" t="inlineStr"/>
+      <c r="I1797" t="inlineStr">
+        <is>
+          <t>Previsto</t>
+        </is>
+      </c>
+      <c r="J1797" t="inlineStr">
+        <is>
+          <t>Ampere</t>
+        </is>
+      </c>
+      <c r="K1797" t="n">
+        <v>20260630</v>
+      </c>
+      <c r="L1797" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="M1797" s="1" t="n">
+        <v>46203</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>